<commit_message>
Fixed ID matching students: uses ID only, but verifies name
</commit_message>
<xml_diff>
--- a/Testing/basic_sequence/workbook_test.xlsx
+++ b/Testing/basic_sequence/workbook_test.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavan Rauch\git\Truancy-Local\Testing\basic_sequence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB7959B-F8C1-42F6-BF5A-121B44990BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8431F5B-4FBD-4A04-94A8-D1A2DFC30BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="step0" sheetId="1" r:id="rId1"/>
-    <sheet name="step1" sheetId="3" r:id="rId2"/>
-    <sheet name="step1same" sheetId="4" r:id="rId3"/>
-    <sheet name="step1diff" sheetId="5" r:id="rId4"/>
+    <sheet name="step0 test" sheetId="6" r:id="rId1"/>
+    <sheet name="step0" sheetId="1" r:id="rId2"/>
+    <sheet name="step1" sheetId="3" r:id="rId3"/>
+    <sheet name="step1same" sheetId="4" r:id="rId4"/>
+    <sheet name="step1diff" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="52">
   <si>
     <t>Last Name</t>
   </si>
@@ -617,6 +618,551 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673F0D56-8560-4A6A-AB03-B01B1AB55396}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P45"/>
+  <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6" customWidth="1"/>
+    <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
+    <col min="8" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="9">
+        <v>117031</v>
+      </c>
+      <c r="D2" s="11">
+        <v>10</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="24">
+        <v>0</v>
+      </c>
+      <c r="I2" s="22">
+        <v>6</v>
+      </c>
+      <c r="J2" s="22">
+        <v>52</v>
+      </c>
+      <c r="K2" s="22">
+        <v>58</v>
+      </c>
+      <c r="L2" s="26">
+        <v>40</v>
+      </c>
+      <c r="M2" s="26">
+        <v>40</v>
+      </c>
+      <c r="N2" s="26">
+        <v>52</v>
+      </c>
+      <c r="O2" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="9">
+        <v>116157</v>
+      </c>
+      <c r="D3" s="11">
+        <v>12</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="24">
+        <v>0</v>
+      </c>
+      <c r="I3" s="22">
+        <v>0</v>
+      </c>
+      <c r="J3" s="22">
+        <v>43.15</v>
+      </c>
+      <c r="K3" s="22">
+        <v>43.15</v>
+      </c>
+      <c r="L3" s="22">
+        <v>23.15</v>
+      </c>
+      <c r="M3" s="22">
+        <v>23.15</v>
+      </c>
+      <c r="N3" s="26">
+        <v>43.15</v>
+      </c>
+      <c r="O3" s="13"/>
+    </row>
+    <row r="4" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="9">
+        <v>115936</v>
+      </c>
+      <c r="D4" s="11">
+        <v>8</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="24">
+        <v>0</v>
+      </c>
+      <c r="I4" s="22">
+        <v>25</v>
+      </c>
+      <c r="J4" s="22">
+        <v>15</v>
+      </c>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22">
+        <v>0</v>
+      </c>
+      <c r="M4" s="22">
+        <v>15</v>
+      </c>
+      <c r="N4" s="22">
+        <v>15</v>
+      </c>
+      <c r="O4" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="9">
+        <v>118245</v>
+      </c>
+      <c r="D5" s="11">
+        <v>7</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="24">
+        <v>0</v>
+      </c>
+      <c r="I5" s="22">
+        <v>79</v>
+      </c>
+      <c r="J5" s="22">
+        <v>0</v>
+      </c>
+      <c r="K5" s="22">
+        <v>79</v>
+      </c>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22">
+        <v>0</v>
+      </c>
+      <c r="N5" s="22">
+        <v>0</v>
+      </c>
+      <c r="O5" s="13"/>
+    </row>
+    <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="9">
+        <v>118678</v>
+      </c>
+      <c r="D6" s="11">
+        <v>9</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="24">
+        <v>0</v>
+      </c>
+      <c r="I6" s="22">
+        <v>30</v>
+      </c>
+      <c r="J6" s="22">
+        <v>10</v>
+      </c>
+      <c r="K6" s="22">
+        <v>40</v>
+      </c>
+      <c r="L6" s="22">
+        <v>0</v>
+      </c>
+      <c r="M6" s="22">
+        <v>10</v>
+      </c>
+      <c r="N6" s="22">
+        <v>10</v>
+      </c>
+      <c r="O6" s="13"/>
+    </row>
+    <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="9">
+        <v>121874</v>
+      </c>
+      <c r="D7" s="11">
+        <v>8</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="24">
+        <v>8.25</v>
+      </c>
+      <c r="I7" s="22">
+        <v>0</v>
+      </c>
+      <c r="J7" s="22">
+        <v>32</v>
+      </c>
+      <c r="K7" s="22">
+        <v>32</v>
+      </c>
+      <c r="L7" s="26">
+        <v>56.33</v>
+      </c>
+      <c r="M7" s="26">
+        <v>56.33</v>
+      </c>
+      <c r="N7" s="22">
+        <v>32</v>
+      </c>
+      <c r="O7" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="P7" s="14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="9">
+        <v>122965</v>
+      </c>
+      <c r="D8" s="11">
+        <v>7</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="24">
+        <v>0</v>
+      </c>
+      <c r="I8" s="22">
+        <v>25</v>
+      </c>
+      <c r="J8" s="22">
+        <v>45</v>
+      </c>
+      <c r="K8" s="22">
+        <v>70</v>
+      </c>
+      <c r="L8" s="22">
+        <v>15</v>
+      </c>
+      <c r="M8" s="22">
+        <v>15</v>
+      </c>
+      <c r="N8" s="26">
+        <v>45</v>
+      </c>
+      <c r="O8" s="15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="17">
+        <v>125674</v>
+      </c>
+      <c r="D9" s="19">
+        <v>9</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="25">
+        <v>0</v>
+      </c>
+      <c r="I9" s="23">
+        <v>13</v>
+      </c>
+      <c r="J9" s="23">
+        <v>55</v>
+      </c>
+      <c r="K9" s="23">
+        <v>35</v>
+      </c>
+      <c r="L9" s="23">
+        <v>55</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="N9" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="O9" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="9"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="13"/>
+    </row>
+    <row r="11" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="9"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
+      <c r="L11" s="22"/>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="13"/>
+    </row>
+    <row r="12" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="H12" s="16"/>
+    </row>
+    <row r="13" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="H13" s="16"/>
+    </row>
+    <row r="14" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="H14" s="16"/>
+    </row>
+    <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="H15" s="16"/>
+    </row>
+    <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="H16" s="16"/>
+    </row>
+    <row r="17" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H17" s="16"/>
+    </row>
+    <row r="18" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H18" s="16"/>
+    </row>
+    <row r="19" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H19" s="16"/>
+    </row>
+    <row r="20" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H20" s="16"/>
+    </row>
+    <row r="21" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H21" s="16"/>
+    </row>
+    <row r="22" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H22" s="16"/>
+    </row>
+    <row r="23" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H23" s="16"/>
+    </row>
+    <row r="24" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H24" s="16"/>
+    </row>
+    <row r="25" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H25" s="16"/>
+    </row>
+    <row r="26" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H26" s="16"/>
+    </row>
+    <row r="27" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H27" s="16"/>
+    </row>
+    <row r="28" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H28" s="16"/>
+    </row>
+    <row r="29" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H29" s="16"/>
+    </row>
+    <row r="30" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H30" s="16"/>
+    </row>
+    <row r="31" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H31" s="16"/>
+    </row>
+    <row r="32" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H32" s="16"/>
+    </row>
+    <row r="33" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H33" s="16"/>
+    </row>
+    <row r="34" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H34" s="16"/>
+    </row>
+    <row r="35" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H35" s="16"/>
+    </row>
+    <row r="36" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H36" s="16"/>
+    </row>
+    <row r="37" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H37" s="16"/>
+    </row>
+    <row r="38" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H38" s="16"/>
+    </row>
+    <row r="39" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H39" s="16"/>
+    </row>
+    <row r="40" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H40" s="16"/>
+    </row>
+    <row r="41" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H41" s="16"/>
+    </row>
+    <row r="42" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H42" s="16"/>
+    </row>
+    <row r="43" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H43" s="16"/>
+    </row>
+    <row r="44" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H44" s="16"/>
+    </row>
+    <row r="45" spans="8:8" ht="15" x14ac:dyDescent="0.25">
+      <c r="H45" s="16"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1161,7 +1707,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{470B75F4-3822-4262-81FF-9A138D10BB04}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1777,7 +2323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96A60C29-17F6-4043-B860-AFE0AE098CC5}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -2393,7 +2939,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE502EA8-8C87-48CA-B9E3-A355F6CA88BA}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>

</xml_diff>

<commit_message>
Handling students missing from report and students missing from sheet
</commit_message>
<xml_diff>
--- a/Testing/basic_sequence/workbook_test.xlsx
+++ b/Testing/basic_sequence/workbook_test.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavan Rauch\git\Truancy-Local\Testing\basic_sequence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71E1531-DFCE-48FA-9ED8-37CD61F40893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE15DE0-72A7-4CE5-AB7E-26BEB8DF2541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="step0 test" sheetId="7" r:id="rId1"/>
+    <sheet name="step0test" sheetId="8" r:id="rId1"/>
     <sheet name="step0" sheetId="1" r:id="rId2"/>
-    <sheet name="step1" sheetId="3" r:id="rId3"/>
+    <sheet name="step1" sheetId="9" r:id="rId3"/>
     <sheet name="step1same" sheetId="4" r:id="rId4"/>
     <sheet name="step1diff" sheetId="5" r:id="rId5"/>
   </sheets>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="55">
   <si>
     <t>Last Name</t>
   </si>
@@ -238,7 +238,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -266,12 +266,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC8C8C8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -303,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -374,10 +368,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -640,11 +630,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{775B543E-04B9-4F3E-B1A1-C58A7F50117F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93028F7D-3C48-46F0-BFF7-CC7FFF17FD71}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
@@ -654,11 +644,11 @@
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
+    <col min="8" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="32.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="90" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -684,13 +674,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>44</v>
@@ -701,11 +691,14 @@
       <c r="N1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>22</v>
       </c>
@@ -724,16 +717,16 @@
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
       <c r="H2" s="24">
-        <v>0</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="I2" s="22">
         <v>6</v>
       </c>
       <c r="J2" s="22">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="K2" s="22">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="L2" s="26">
         <v>40</v>
@@ -744,11 +737,14 @@
       <c r="N2" s="26">
         <v>52</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="26">
+        <v>62</v>
+      </c>
+      <c r="P2" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>20</v>
       </c>
@@ -770,13 +766,13 @@
         <v>0</v>
       </c>
       <c r="I3" s="22">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J3" s="22">
-        <v>43.15</v>
+        <v>50.15</v>
       </c>
       <c r="K3" s="22">
-        <v>43.15</v>
+        <v>56.15</v>
       </c>
       <c r="L3" s="22">
         <v>23.15</v>
@@ -787,9 +783,12 @@
       <c r="N3" s="26">
         <v>43.15</v>
       </c>
-      <c r="O3" s="13"/>
-    </row>
-    <row r="4" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O3" s="26">
+        <v>50.15</v>
+      </c>
+      <c r="P3" s="13"/>
+    </row>
+    <row r="4" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>18</v>
       </c>
@@ -811,12 +810,14 @@
         <v>0</v>
       </c>
       <c r="I4" s="22">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="J4" s="22">
-        <v>15</v>
-      </c>
-      <c r="K4" s="22"/>
+        <v>0</v>
+      </c>
+      <c r="K4" s="22">
+        <v>42</v>
+      </c>
       <c r="L4" s="22">
         <v>0</v>
       </c>
@@ -826,11 +827,14 @@
       <c r="N4" s="22">
         <v>15</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="27">
+        <v>0</v>
+      </c>
+      <c r="P4" s="13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>24</v>
       </c>
@@ -852,13 +856,13 @@
         <v>0</v>
       </c>
       <c r="I5" s="22">
-        <v>79</v>
+        <v>85.75</v>
       </c>
       <c r="J5" s="22">
         <v>0</v>
       </c>
       <c r="K5" s="22">
-        <v>79</v>
+        <v>85.75</v>
       </c>
       <c r="L5" s="22"/>
       <c r="M5" s="22">
@@ -867,9 +871,12 @@
       <c r="N5" s="22">
         <v>0</v>
       </c>
-      <c r="O5" s="13"/>
-    </row>
-    <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O5" s="27">
+        <v>0</v>
+      </c>
+      <c r="P5" s="13"/>
+    </row>
+    <row r="6" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>26</v>
       </c>
@@ -908,9 +915,12 @@
       <c r="N6" s="22">
         <v>10</v>
       </c>
-      <c r="O6" s="13"/>
-    </row>
-    <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O6" s="27">
+        <v>10</v>
+      </c>
+      <c r="P6" s="13"/>
+    </row>
+    <row r="7" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>28</v>
       </c>
@@ -949,14 +959,17 @@
       <c r="N7" s="22">
         <v>32</v>
       </c>
-      <c r="O7" s="13" t="s">
+      <c r="O7" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="P7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="P7" s="14" t="s">
+      <c r="Q7" s="14" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>30</v>
       </c>
@@ -981,10 +994,10 @@
         <v>25</v>
       </c>
       <c r="J8" s="22">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="K8" s="22">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="L8" s="22">
         <v>15</v>
@@ -995,11 +1008,14 @@
       <c r="N8" s="26">
         <v>45</v>
       </c>
-      <c r="O8" s="15" t="s">
+      <c r="O8" s="27">
+        <v>15</v>
+      </c>
+      <c r="P8" s="15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>32</v>
       </c>
@@ -1038,57 +1054,102 @@
       <c r="N9" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="O9" s="21" t="s">
+      <c r="O9" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="P9" s="21" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="10"/>
+    <row r="10" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="3">
+        <v>119789</v>
+      </c>
+      <c r="D10" s="11">
+        <v>11</v>
+      </c>
+      <c r="E10" s="10">
+        <v>4</v>
+      </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
+      <c r="H10" s="24">
+        <v>0</v>
+      </c>
+      <c r="I10" s="22">
+        <v>20</v>
+      </c>
+      <c r="J10" s="22">
+        <v>35</v>
+      </c>
+      <c r="K10" s="22">
+        <v>55</v>
+      </c>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
       <c r="N10" s="22"/>
-      <c r="O10" s="13"/>
-    </row>
-    <row r="11" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="10"/>
+      <c r="O10" s="22">
+        <v>35</v>
+      </c>
+      <c r="P10" s="13"/>
+    </row>
+    <row r="11" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="3">
+        <v>120451</v>
+      </c>
+      <c r="D11" s="11">
+        <v>10</v>
+      </c>
+      <c r="E11" s="10">
+        <v>5</v>
+      </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
+      <c r="H11" s="24">
+        <v>0</v>
+      </c>
+      <c r="I11" s="22">
+        <v>15</v>
+      </c>
+      <c r="J11" s="22">
+        <v>40</v>
+      </c>
+      <c r="K11" s="22">
+        <v>65</v>
+      </c>
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
-      <c r="O11" s="13"/>
-    </row>
-    <row r="12" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O11" s="26">
+        <v>40</v>
+      </c>
+      <c r="P11" s="13"/>
+    </row>
+    <row r="12" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H16" s="16"/>
     </row>
     <row r="17" spans="8:8" ht="15" x14ac:dyDescent="0.25">
@@ -1730,11 +1791,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{470B75F4-3822-4262-81FF-9A138D10BB04}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E148BF83-6447-4D72-A8FE-C2168CADDB3C}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
@@ -1744,11 +1805,11 @@
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="32.28515625" style="2" customWidth="1"/>
+    <col min="8" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="32.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="90" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1774,13 +1835,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>44</v>
@@ -1794,14 +1855,11 @@
       <c r="O1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="P1" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>22</v>
       </c>
@@ -1843,14 +1901,11 @@
       <c r="O2" s="26">
         <v>62</v>
       </c>
-      <c r="P2" s="26">
-        <v>62</v>
-      </c>
-      <c r="Q2" s="13" t="s">
+      <c r="P2" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>20</v>
       </c>
@@ -1892,12 +1947,9 @@
       <c r="O3" s="26">
         <v>50.15</v>
       </c>
-      <c r="P3" s="26">
-        <v>50.15</v>
-      </c>
-      <c r="Q3" s="13"/>
-    </row>
-    <row r="4" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="P3" s="13"/>
+    </row>
+    <row r="4" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>18</v>
       </c>
@@ -1939,14 +1991,11 @@
       <c r="O4" s="22">
         <v>0</v>
       </c>
-      <c r="P4" s="27">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="13" t="s">
+      <c r="P4" s="13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>24</v>
       </c>
@@ -1986,12 +2035,9 @@
       <c r="O5" s="22">
         <v>0</v>
       </c>
-      <c r="P5" s="27">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="13"/>
-    </row>
-    <row r="6" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="P5" s="13"/>
+    </row>
+    <row r="6" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>26</v>
       </c>
@@ -2033,12 +2079,9 @@
       <c r="O6" s="22">
         <v>10</v>
       </c>
-      <c r="P6" s="27">
-        <v>10</v>
-      </c>
-      <c r="Q6" s="13"/>
-    </row>
-    <row r="7" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="P6" s="13"/>
+    </row>
+    <row r="7" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>28</v>
       </c>
@@ -2080,15 +2123,14 @@
       <c r="O7" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="13" t="s">
+      <c r="P7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="R7" s="14" t="s">
+      <c r="Q7" s="14" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>30</v>
       </c>
@@ -2130,14 +2172,11 @@
       <c r="O8" s="22">
         <v>15</v>
       </c>
-      <c r="P8" s="27">
-        <v>15</v>
-      </c>
-      <c r="Q8" s="15" t="s">
+      <c r="P8" s="15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>32</v>
       </c>
@@ -2179,12 +2218,11 @@
       <c r="O9" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="21" t="s">
+      <c r="P9" s="21" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>47</v>
       </c>
@@ -2220,12 +2258,9 @@
       <c r="O10" s="22">
         <v>35</v>
       </c>
-      <c r="P10" s="27">
-        <v>35</v>
-      </c>
-      <c r="Q10" s="13"/>
-    </row>
-    <row r="11" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="P10" s="13"/>
+    </row>
+    <row r="11" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>49</v>
       </c>
@@ -2261,146 +2296,109 @@
       <c r="O11" s="26">
         <v>40</v>
       </c>
-      <c r="P11" s="26">
-        <v>40</v>
-      </c>
-      <c r="Q11" s="13"/>
-    </row>
-    <row r="12" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="P11" s="13"/>
+    </row>
+    <row r="12" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H12" s="16"/>
-      <c r="P12" s="28"/>
-    </row>
-    <row r="13" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H13" s="16"/>
-      <c r="P13" s="28"/>
-    </row>
-    <row r="14" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H14" s="16"/>
-      <c r="P14" s="28"/>
-    </row>
-    <row r="15" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H15" s="16"/>
-      <c r="P15" s="28"/>
-    </row>
-    <row r="16" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:17" ht="15" x14ac:dyDescent="0.25">
       <c r="H16" s="16"/>
-      <c r="P16" s="28"/>
-    </row>
-    <row r="17" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H17" s="16"/>
-      <c r="P17" s="28"/>
-    </row>
-    <row r="18" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H18" s="16"/>
-      <c r="P18" s="28"/>
-    </row>
-    <row r="19" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H19" s="16"/>
-      <c r="P19" s="28"/>
-    </row>
-    <row r="20" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H20" s="16"/>
-      <c r="P20" s="28"/>
-    </row>
-    <row r="21" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H21" s="16"/>
-      <c r="P21" s="28"/>
-    </row>
-    <row r="22" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H22" s="16"/>
-      <c r="P22" s="28"/>
-    </row>
-    <row r="23" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H23" s="16"/>
-      <c r="P23" s="28"/>
-    </row>
-    <row r="24" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H24" s="16"/>
-      <c r="P24" s="28"/>
-    </row>
-    <row r="25" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H25" s="16"/>
-      <c r="P25" s="28"/>
-    </row>
-    <row r="26" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H26" s="16"/>
-      <c r="P26" s="28"/>
-    </row>
-    <row r="27" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H27" s="16"/>
-      <c r="P27" s="28"/>
-    </row>
-    <row r="28" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H28" s="16"/>
-      <c r="P28" s="28"/>
-    </row>
-    <row r="29" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H29" s="16"/>
-      <c r="P29" s="28"/>
-    </row>
-    <row r="30" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H30" s="16"/>
-      <c r="P30" s="28"/>
-    </row>
-    <row r="31" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H31" s="16"/>
-      <c r="P31" s="28"/>
-    </row>
-    <row r="32" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H32" s="16"/>
-      <c r="P32" s="28"/>
-    </row>
-    <row r="33" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H33" s="16"/>
-      <c r="P33" s="28"/>
-    </row>
-    <row r="34" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H34" s="16"/>
-      <c r="P34" s="28"/>
-    </row>
-    <row r="35" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H35" s="16"/>
-      <c r="P35" s="28"/>
-    </row>
-    <row r="36" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H36" s="16"/>
-      <c r="P36" s="28"/>
-    </row>
-    <row r="37" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H37" s="16"/>
-      <c r="P37" s="28"/>
-    </row>
-    <row r="38" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H38" s="16"/>
-      <c r="P38" s="28"/>
-    </row>
-    <row r="39" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H39" s="16"/>
-      <c r="P39" s="28"/>
-    </row>
-    <row r="40" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="16"/>
-      <c r="P40" s="28"/>
-    </row>
-    <row r="41" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H41" s="16"/>
-      <c r="P41" s="28"/>
-    </row>
-    <row r="42" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H42" s="16"/>
-      <c r="P42" s="28"/>
-    </row>
-    <row r="43" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H43" s="16"/>
-      <c r="P43" s="28"/>
-    </row>
-    <row r="44" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H44" s="16"/>
-      <c r="P44" s="28"/>
-    </row>
-    <row r="45" spans="8:16" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="8:8" ht="15" x14ac:dyDescent="0.25">
       <c r="H45" s="16"/>
-      <c r="P45" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
More useful status box
</commit_message>
<xml_diff>
--- a/Testing/basic_sequence/workbook_test.xlsx
+++ b/Testing/basic_sequence/workbook_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavan Rauch\git\Truancy-Local\Testing\basic_sequence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE15DE0-72A7-4CE5-AB7E-26BEB8DF2541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B19279-91C5-497B-9452-E92EF5457013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="52">
   <si>
     <t>Last Name</t>
   </si>
@@ -185,15 +185,6 @@
   </si>
   <si>
     <t>1/28/24 Total Absences (minus suspension hours)</t>
-  </si>
-  <si>
-    <t>03/05/2026 Excused Absences</t>
-  </si>
-  <si>
-    <t>03/05/2026 Unexcused Absences</t>
-  </si>
-  <si>
-    <t>03/05/2026 Total Absences (minus suspension hours)</t>
   </si>
 </sst>
 </file>
@@ -297,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -365,9 +356,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -634,7 +622,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q45"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
@@ -644,11 +632,11 @@
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="32.28515625" style="2" customWidth="1"/>
+    <col min="8" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -674,13 +662,13 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>44</v>
@@ -691,14 +679,11 @@
       <c r="N1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="P1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>22</v>
       </c>
@@ -717,16 +702,16 @@
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
       <c r="H2" s="24">
-        <v>19.399999999999999</v>
+        <v>0</v>
       </c>
       <c r="I2" s="22">
         <v>6</v>
       </c>
       <c r="J2" s="22">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K2" s="22">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="L2" s="26">
         <v>40</v>
@@ -737,14 +722,11 @@
       <c r="N2" s="26">
         <v>52</v>
       </c>
-      <c r="O2" s="26">
-        <v>62</v>
-      </c>
-      <c r="P2" s="13" t="s">
+      <c r="O2" s="13" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>20</v>
       </c>
@@ -766,13 +748,13 @@
         <v>0</v>
       </c>
       <c r="I3" s="22">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J3" s="22">
-        <v>50.15</v>
+        <v>43.15</v>
       </c>
       <c r="K3" s="22">
-        <v>56.15</v>
+        <v>43.15</v>
       </c>
       <c r="L3" s="22">
         <v>23.15</v>
@@ -783,12 +765,9 @@
       <c r="N3" s="26">
         <v>43.15</v>
       </c>
-      <c r="O3" s="26">
-        <v>50.15</v>
-      </c>
-      <c r="P3" s="13"/>
-    </row>
-    <row r="4" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="O3" s="13"/>
+    </row>
+    <row r="4" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>18</v>
       </c>
@@ -810,14 +789,12 @@
         <v>0</v>
       </c>
       <c r="I4" s="22">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="J4" s="22">
-        <v>0</v>
-      </c>
-      <c r="K4" s="22">
-        <v>42</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="K4" s="22"/>
       <c r="L4" s="22">
         <v>0</v>
       </c>
@@ -827,14 +804,11 @@
       <c r="N4" s="22">
         <v>15</v>
       </c>
-      <c r="O4" s="27">
-        <v>0</v>
-      </c>
-      <c r="P4" s="13" t="s">
+      <c r="O4" s="13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>24</v>
       </c>
@@ -856,13 +830,13 @@
         <v>0</v>
       </c>
       <c r="I5" s="22">
-        <v>85.75</v>
+        <v>79</v>
       </c>
       <c r="J5" s="22">
         <v>0</v>
       </c>
       <c r="K5" s="22">
-        <v>85.75</v>
+        <v>79</v>
       </c>
       <c r="L5" s="22"/>
       <c r="M5" s="22">
@@ -871,12 +845,9 @@
       <c r="N5" s="22">
         <v>0</v>
       </c>
-      <c r="O5" s="27">
-        <v>0</v>
-      </c>
-      <c r="P5" s="13"/>
-    </row>
-    <row r="6" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="O5" s="13"/>
+    </row>
+    <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>26</v>
       </c>
@@ -915,12 +886,9 @@
       <c r="N6" s="22">
         <v>10</v>
       </c>
-      <c r="O6" s="27">
-        <v>10</v>
-      </c>
-      <c r="P6" s="13"/>
-    </row>
-    <row r="7" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="O6" s="13"/>
+    </row>
+    <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>28</v>
       </c>
@@ -959,17 +927,14 @@
       <c r="N7" s="22">
         <v>32</v>
       </c>
-      <c r="O7" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P7" s="13" t="s">
+      <c r="O7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="Q7" s="14" t="s">
+      <c r="P7" s="14" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>30</v>
       </c>
@@ -994,10 +959,10 @@
         <v>25</v>
       </c>
       <c r="J8" s="22">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="K8" s="22">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="L8" s="22">
         <v>15</v>
@@ -1008,14 +973,11 @@
       <c r="N8" s="26">
         <v>45</v>
       </c>
-      <c r="O8" s="27">
-        <v>15</v>
-      </c>
-      <c r="P8" s="15" t="s">
+      <c r="O8" s="15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>32</v>
       </c>
@@ -1054,102 +1016,57 @@
       <c r="N9" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="O9" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="P9" s="21" t="s">
+      <c r="O9" s="21" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="3">
-        <v>119789</v>
-      </c>
-      <c r="D10" s="11">
-        <v>11</v>
-      </c>
-      <c r="E10" s="10">
-        <v>4</v>
-      </c>
+    <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A10" s="9"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="10"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="24">
-        <v>0</v>
-      </c>
-      <c r="I10" s="22">
-        <v>20</v>
-      </c>
-      <c r="J10" s="22">
-        <v>35</v>
-      </c>
-      <c r="K10" s="22">
-        <v>55</v>
-      </c>
+      <c r="H10" s="24"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
       <c r="N10" s="22"/>
-      <c r="O10" s="22">
-        <v>35</v>
-      </c>
-      <c r="P10" s="13"/>
-    </row>
-    <row r="11" spans="1:17" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="3">
-        <v>120451</v>
-      </c>
-      <c r="D11" s="11">
-        <v>10</v>
-      </c>
-      <c r="E11" s="10">
-        <v>5</v>
-      </c>
+      <c r="O10" s="13"/>
+    </row>
+    <row r="11" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="9"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="10"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
-      <c r="H11" s="24">
-        <v>0</v>
-      </c>
-      <c r="I11" s="22">
-        <v>15</v>
-      </c>
-      <c r="J11" s="22">
-        <v>40</v>
-      </c>
-      <c r="K11" s="22">
-        <v>65</v>
-      </c>
+      <c r="H11" s="24"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="22"/>
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
-      <c r="O11" s="26">
-        <v>40</v>
-      </c>
-      <c r="P11" s="13"/>
-    </row>
-    <row r="12" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+      <c r="O11" s="13"/>
+    </row>
+    <row r="12" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="H12" s="16"/>
     </row>
-    <row r="13" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="H13" s="16"/>
     </row>
-    <row r="14" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="H14" s="16"/>
     </row>
-    <row r="15" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="H15" s="16"/>
     </row>
-    <row r="16" spans="1:17" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="H16" s="16"/>
     </row>
     <row r="17" spans="8:8" ht="15" x14ac:dyDescent="0.25">

</xml_diff>